<commit_message>
fix(#334): clarifie la sous-extension methodCollection et distingue CV / Appli CV
Ajoute un ^definition à extension[methodCollection] et à chaque concept du
CodeSystem fr-core-cs-method-collection, en référençant le RNIV §4.3, pour
lever l'ambiguïté entre canal de capture (methodCollection), statut de
confiance (identityStatus) et pièce justificative (validationMode).

Ajoute le code AV (Application carte Vitale) pour distinguer explicitement
la carte Vitale physique de sa version dématérialisée (RNIV §4.3.4), et
corrige la Description du ValueSet copiée-collée depuis validationMode.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com> 5c5b88cef87af34aac3c7ba1f7778688114b73c8
</commit_message>
<xml_diff>
--- a/fix/issue-298-identity-status-rniv/ig/CodeSystem-fr-core-cs-method-collection.xlsx
+++ b/fix/issue-298-identity-status-rniv/ig/CodeSystem-fr-core-cs-method-collection.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="61">
   <si>
     <t>Property</t>
   </si>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-08-10T13:14:57+00:00</t>
+    <t>2026-08-10T13:29:34+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -126,7 +126,7 @@
     <t>Count</t>
   </si>
   <si>
-    <t>5</t>
+    <t>6</t>
   </si>
   <si>
     <t>Level</t>
@@ -150,16 +150,25 @@
     <t>Saisie manuelle</t>
   </si>
   <si>
+    <t>Saisie manuelle des traits d'identité, sans lecture de la carte Vitale ni interrogation du téléservice INSi (RNIV §4.3.3).</t>
+  </si>
+  <si>
     <t>CV</t>
   </si>
   <si>
-    <t>Carte vitale</t>
+    <t>Carte Vitale</t>
+  </si>
+  <si>
+    <t>Lecture de la carte Vitale physique de l'usager, permettant l'interrogation du téléservice INSi par ce canal (RNIV §4.3.2).</t>
   </si>
   <si>
     <t>INSI</t>
   </si>
   <si>
-    <t>Téléservice INSI</t>
+    <t>Téléservice INSi</t>
+  </si>
+  <si>
+    <t>Interrogation directe du téléservice INSi par saisie des traits d'identité, sans lecture de la carte Vitale (RNIV §4.3.3).</t>
   </si>
   <si>
     <t>CB</t>
@@ -168,10 +177,25 @@
     <t>Code à barre</t>
   </si>
   <si>
+    <t>Import de l'identité par scan du Datamatrix INS figurant sur un document de santé déjà porteur d'une identité qualifiée (Guide d'implémentation INS, EXI REC 02).</t>
+  </si>
+  <si>
     <t>RFID</t>
   </si>
   <si>
     <t>Puce RFID</t>
+  </si>
+  <si>
+    <t>Lecture d'une puce RFID (ex. bracelet patient) ; canal local de traçabilité, non défini par le RNIV.</t>
+  </si>
+  <si>
+    <t>AV</t>
+  </si>
+  <si>
+    <t>Application carte Vitale</t>
+  </si>
+  <si>
+    <t>Obtention directe de l'INS par scan du QR code ou lecture NFC de l'Application carte Vitale (RNIV §4.3.4) ; l'identité ainsi obtenue est considérée comme qualifiée.</t>
   </si>
 </sst>
 </file>
@@ -489,7 +513,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -517,7 +541,7 @@
         <v>44</v>
       </c>
       <c r="D2" t="s" s="2">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="3">
@@ -525,13 +549,13 @@
         <v>42</v>
       </c>
       <c r="B3" t="s" s="2">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C3" t="s" s="2">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D3" t="s" s="2">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="4">
@@ -539,13 +563,13 @@
         <v>42</v>
       </c>
       <c r="B4" t="s" s="2">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="C4" t="s" s="2">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="D4" t="s" s="2">
-        <v>48</v>
+        <v>51</v>
       </c>
     </row>
     <row r="5">
@@ -553,13 +577,13 @@
         <v>42</v>
       </c>
       <c r="B5" t="s" s="2">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="C5" t="s" s="2">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="D5" t="s" s="2">
-        <v>50</v>
+        <v>54</v>
       </c>
     </row>
     <row r="6">
@@ -567,13 +591,27 @@
         <v>42</v>
       </c>
       <c r="B6" t="s" s="2">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="C6" t="s" s="2">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="D6" t="s" s="2">
-        <v>52</v>
+        <v>57</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s" s="2">
+        <v>42</v>
+      </c>
+      <c r="B7" t="s" s="2">
+        <v>58</v>
+      </c>
+      <c r="C7" t="s" s="2">
+        <v>59</v>
+      </c>
+      <c r="D7" t="s" s="2">
+        <v>60</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix(#334): déplace les références RNIV en commentaires FSH et précise la version du référentiel
Les références "(RNIV §4.3.x)" étaient embarquées dans les ^definition et
display, couplant fortement le texte publié à une numérotation de
paragraphe susceptible de changer d'une version à l'autre du RNIV. Elles
sont déplacées en commentaires FSH, avec la version exacte du référentiel
citée (RNIV 1 - Principes communs v2.0, Guide d'implémentation INS v3.0,
décembre 2024). Réordonne aussi ^short de methodCollection (français puis
anglais), conformément à la convention du fichier.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com> fd14905567cb42b4f3a2b47b51027da18f4dc0c5
</commit_message>
<xml_diff>
--- a/fix/issue-298-identity-status-rniv/ig/CodeSystem-fr-core-cs-method-collection.xlsx
+++ b/fix/issue-298-identity-status-rniv/ig/CodeSystem-fr-core-cs-method-collection.xlsx
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-08-10T13:29:34+00:00</t>
+    <t>2026-08-10T13:33:35+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -150,7 +150,7 @@
     <t>Saisie manuelle</t>
   </si>
   <si>
-    <t>Saisie manuelle des traits d'identité, sans lecture de la carte Vitale ni interrogation du téléservice INSi (RNIV §4.3.3).</t>
+    <t>Saisie manuelle des traits d'identité, sans lecture de la carte Vitale ni interrogation du téléservice INSi.</t>
   </si>
   <si>
     <t>CV</t>
@@ -159,7 +159,7 @@
     <t>Carte Vitale</t>
   </si>
   <si>
-    <t>Lecture de la carte Vitale physique de l'usager, permettant l'interrogation du téléservice INSi par ce canal (RNIV §4.3.2).</t>
+    <t>Lecture de la carte Vitale physique de l'usager, permettant l'interrogation du téléservice INSi par ce canal.</t>
   </si>
   <si>
     <t>INSI</t>
@@ -168,7 +168,7 @@
     <t>Téléservice INSi</t>
   </si>
   <si>
-    <t>Interrogation directe du téléservice INSi par saisie des traits d'identité, sans lecture de la carte Vitale (RNIV §4.3.3).</t>
+    <t>Interrogation directe du téléservice INSi par saisie des traits d'identité, sans lecture de la carte Vitale.</t>
   </si>
   <si>
     <t>CB</t>
@@ -177,7 +177,7 @@
     <t>Code à barre</t>
   </si>
   <si>
-    <t>Import de l'identité par scan du Datamatrix INS figurant sur un document de santé déjà porteur d'une identité qualifiée (Guide d'implémentation INS, EXI REC 02).</t>
+    <t>Import de l'identité par scan du Datamatrix INS figurant sur un document de santé déjà porteur d'une identité qualifiée.</t>
   </si>
   <si>
     <t>RFID</t>
@@ -195,7 +195,7 @@
     <t>Application carte Vitale</t>
   </si>
   <si>
-    <t>Obtention directe de l'INS par scan du QR code ou lecture NFC de l'Application carte Vitale (RNIV §4.3.4) ; l'identité ainsi obtenue est considérée comme qualifiée.</t>
+    <t>Obtention directe de l'INS par scan du QR code ou lecture NFC de l'Application carte Vitale ; l'identité ainsi obtenue est considérée comme qualifiée.</t>
   </si>
 </sst>
 </file>

</xml_diff>